<commit_message>
Phase 1 구현: InputGateway/DegradedStateManager/SensorFaultGate (TDD)
branch coverage 100%, lizard/pylint 품질지표 통과.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -818,12 +818,6 @@
           <t>ApproachRiskPolicy</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -841,12 +835,26 @@
           <t>InputGateway, DegradedStateManager</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-001 (Phase1 기반모듈)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>src/vjecl/input_gateway.py, src/vjecl/degraded_state_manager.py</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>tests/test_input_gateway.py, tests/test_degraded_state_manager.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -864,12 +872,26 @@
           <t>SensorFaultGate</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-001 (Phase1 기반모듈)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>src/vjecl/sensor_fault_gate.py</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>tests/test_sensor_fault_gate.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -887,12 +909,6 @@
           <t>DriverCommandPolicy</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -910,12 +926,6 @@
           <t>AutoLockPolicy</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -933,12 +943,6 @@
           <t>ApproachRiskPolicy(override)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -956,12 +960,6 @@
           <t>OutputMapper</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -979,12 +977,6 @@
           <t>ForcedReleasePolicy</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1002,12 +994,6 @@
           <t>IsofixLockPolicy</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1025,12 +1011,6 @@
           <t>IgnitionOffPolicy</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1048,12 +1028,6 @@
           <t>PriorityArbiter(순수함수/결정론)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1071,12 +1045,6 @@
           <t>EventLogStore</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1089,14 +1057,9 @@
           <t>SWR-019</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="24"/>
+    <row r="25"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A5:I5"/>

</xml_diff>

<commit_message>
Phase 1 구현: InputGateway/DegradedStateManager/SensorFaultGate (TDD) (#6)
branch coverage 100%, lizard/pylint 품질지표 통과.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -610,7 +610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -818,12 +818,6 @@
           <t>ApproachRiskPolicy</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -841,12 +835,26 @@
           <t>InputGateway, DegradedStateManager</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-001 (Phase1 기반모듈)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>src/vjecl/input_gateway.py, src/vjecl/degraded_state_manager.py</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>tests/test_input_gateway.py, tests/test_degraded_state_manager.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -864,12 +872,26 @@
           <t>SensorFaultGate</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-001 (Phase1 기반모듈)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>src/vjecl/sensor_fault_gate.py</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>tests/test_sensor_fault_gate.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -887,12 +909,6 @@
           <t>DriverCommandPolicy</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -910,12 +926,6 @@
           <t>AutoLockPolicy</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -933,12 +943,6 @@
           <t>ApproachRiskPolicy(override)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -956,12 +960,6 @@
           <t>OutputMapper</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -979,12 +977,6 @@
           <t>ForcedReleasePolicy</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1002,12 +994,6 @@
           <t>IsofixLockPolicy</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1025,12 +1011,6 @@
           <t>IgnitionOffPolicy</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1048,12 +1028,6 @@
           <t>PriorityArbiter(순수함수/결정론)</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1071,12 +1045,6 @@
           <t>EventLogStore</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1089,14 +1057,9 @@
           <t>SWR-019</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="24"/>
+    <row r="25"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A5:I5"/>

</xml_diff>

<commit_message>
Phase 1 통합시험: InputGateway/DegradedStateManager/SensorFaultGate
함수커버리지 100%, 콜커버리지 100%. call coverage 측정을 위해
input_gateway.normalize()를 지역변수로 분리.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -850,6 +850,11 @@
           <t>tests/test_input_gateway.py, tests/test_degraded_state_manager.py (TDD)</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>IT-P1-01~04 (ENG-SWE5-002/003)</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>branch coverage 100%</t>
@@ -885,6 +890,11 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>tests/test_sensor_fault_gate.py (TDD)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>IT-P1-01~04 (ENG-SWE5-002/003)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">

</xml_diff>

<commit_message>
Phase 1 통합시험: InputGateway/DegradedStateManager/SensorFaultGate (#7)
* Phase 1 통합시험: InputGateway/DegradedStateManager/SensorFaultGate

함수커버리지 100%, 콜커버리지 100%. call coverage 측정을 위해
input_gateway.normalize()를 지역변수로 분리.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* CI 품질지표 수정: 테스트 픽스처 중복 제거 (tests/fixtures.py)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -850,6 +850,11 @@
           <t>tests/test_input_gateway.py, tests/test_degraded_state_manager.py (TDD)</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>IT-P1-01~04 (ENG-SWE5-002/003)</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>branch coverage 100%</t>
@@ -885,6 +890,11 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>tests/test_sensor_fault_gate.py (TDD)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>IT-P1-01~04 (ENG-SWE5-002/003)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">

</xml_diff>

<commit_message>
Phase 2 구현: CrashReleasePolicy/ApproachRiskPolicy (TDD)
branch coverage 100%, 34개 테스트 전부 통과. 품질지표(lizard/pylint/radon) 통과.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -795,12 +795,28 @@
           <t>CrashReleasePolicy</t>
         </is>
       </c>
-      <c r="D10" s="42" t="inlineStr"/>
-      <c r="E10" s="42" t="inlineStr"/>
-      <c r="F10" s="42" t="inlineStr"/>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-002 (Phase2)</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/crash_release_policy.py</t>
+        </is>
+      </c>
+      <c r="F10" s="42" t="inlineStr">
+        <is>
+          <t>tests/test_crash_release_policy.py (TDD)</t>
+        </is>
+      </c>
       <c r="G10" s="42" t="inlineStr"/>
       <c r="H10" s="42" t="inlineStr"/>
-      <c r="I10" s="42" t="inlineStr"/>
+      <c r="I10" s="42" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -818,6 +834,26 @@
           <t>ApproachRiskPolicy</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-002 (Phase2)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/approach_risk_policy.py</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>tests/test_approach_risk_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -951,6 +987,26 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>ApproachRiskPolicy(override)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-002 (Phase2, override 로직)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/approach_risk_policy.py</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>tests/test_approach_risk_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 2 구현: CrashReleasePolicy/ApproachRiskPolicy (TDD) (#10)
branch coverage 100%, 34개 테스트 전부 통과. 품질지표(lizard/pylint/radon) 통과.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -795,12 +795,28 @@
           <t>CrashReleasePolicy</t>
         </is>
       </c>
-      <c r="D10" s="42" t="inlineStr"/>
-      <c r="E10" s="42" t="inlineStr"/>
-      <c r="F10" s="42" t="inlineStr"/>
+      <c r="D10" s="42" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-002 (Phase2)</t>
+        </is>
+      </c>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/crash_release_policy.py</t>
+        </is>
+      </c>
+      <c r="F10" s="42" t="inlineStr">
+        <is>
+          <t>tests/test_crash_release_policy.py (TDD)</t>
+        </is>
+      </c>
       <c r="G10" s="42" t="inlineStr"/>
       <c r="H10" s="42" t="inlineStr"/>
-      <c r="I10" s="42" t="inlineStr"/>
+      <c r="I10" s="42" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -818,6 +834,26 @@
           <t>ApproachRiskPolicy</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-002 (Phase2)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/approach_risk_policy.py</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>tests/test_approach_risk_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -951,6 +987,26 @@
       <c r="C16" t="inlineStr">
         <is>
           <t>ApproachRiskPolicy(override)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-002 (Phase2, override 로직)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/approach_risk_policy.py</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>tests/test_approach_risk_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 구현: ForcedReleasePolicy/IsofixLockPolicy/IgnitionOffPolicy (TDD)
branch coverage 100%, 50개 테스트 전부 통과. 품질지표 통과.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -1057,6 +1057,26 @@
           <t>ForcedReleasePolicy</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-003 (Phase3)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/forced_release_policy.py</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>tests/test_forced_release_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1074,6 +1094,26 @@
           <t>IsofixLockPolicy</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-003 (Phase3)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/isofix_lock_policy.py</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>tests/test_isofix_lock_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1089,6 +1129,26 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>IgnitionOffPolicy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-003 (Phase3)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/ignition_off_policy.py</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>tests/test_ignition_off_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Phase 3 구현: ForcedReleasePolicy/IsofixLockPolicy/IgnitionOffPolicy (TDD) (#14)
branch coverage 100%, 50개 테스트 전부 통과. 품질지표 통과.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
+++ b/02_Tier/02_WorkProduct/doc/engineering/Traceability/ENG-TRC-001_양방향 요구사항 추적 매트릭스.xlsx
@@ -1057,6 +1057,26 @@
           <t>ForcedReleasePolicy</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-003 (Phase3)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/forced_release_policy.py</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>tests/test_forced_release_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1074,6 +1094,26 @@
           <t>IsofixLockPolicy</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-003 (Phase3)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/isofix_lock_policy.py</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>tests/test_isofix_lock_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1089,6 +1129,26 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>IgnitionOffPolicy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ENG-SWE3-003 (Phase3)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>src/vjecl/policies/ignition_off_policy.py</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>tests/test_ignition_off_policy.py (TDD)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>branch coverage 100%</t>
         </is>
       </c>
     </row>

</xml_diff>